<commit_message>
Automatically guesses the version if student left version blank
</commit_message>
<xml_diff>
--- a/All.xlsx
+++ b/All.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\souri\Dropbox\2018-Summer\PHYS 1601\test3\2018-Su\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\souri\Dropbox\Machinegrading\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F83C0DDC-BF75-4962-BC4A-D730F268FBE2}" xr6:coauthVersionLast="33" xr6:coauthVersionMax="33" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74969708-45D5-40E9-97F0-DFCA720BCBF1}" xr6:coauthVersionLast="33" xr6:coauthVersionMax="33" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" xr2:uid="{55B9AD52-30FB-4BC0-874F-7C9A458412C5}"/>
   </bookViews>
@@ -70,18 +70,12 @@
     <t>HAN KARIN</t>
   </si>
   <si>
-    <t>011024102134040</t>
-  </si>
-  <si>
     <t>1015</t>
   </si>
   <si>
     <t>HENRY NICHOLAS</t>
   </si>
   <si>
-    <t>420224033434021</t>
-  </si>
-  <si>
     <t>1002</t>
   </si>
   <si>
@@ -206,6 +200,12 @@
   </si>
   <si>
     <t>430244011141021</t>
+  </si>
+  <si>
+    <t>42022403343402</t>
+  </si>
+  <si>
+    <t>0110241 21 4040</t>
   </si>
 </sst>
 </file>
@@ -600,183 +600,183 @@
         <v>7</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
makes a list of all students that didn't enter test versions
</commit_message>
<xml_diff>
--- a/All.xlsx
+++ b/All.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\souri\Dropbox\Machinegrading\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74969708-45D5-40E9-97F0-DFCA720BCBF1}" xr6:coauthVersionLast="33" xr6:coauthVersionMax="33" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EAEF999-9803-4882-BED4-033BE002D23D}" xr6:coauthVersionLast="33" xr6:coauthVersionMax="33" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" xr2:uid="{55B9AD52-30FB-4BC0-874F-7C9A458412C5}"/>
   </bookViews>
@@ -85,9 +85,6 @@
     <t>334310202024403</t>
   </si>
   <si>
-    <t>1018</t>
-  </si>
-  <si>
     <t>MUEZZINOGLU MINE</t>
   </si>
   <si>
@@ -118,18 +115,9 @@
     <t>DIBBLE HANNAH</t>
   </si>
   <si>
-    <t>334310202224403</t>
-  </si>
-  <si>
-    <t>1017</t>
-  </si>
-  <si>
     <t>MATHUR DIYA</t>
   </si>
   <si>
-    <t>403020044031422</t>
-  </si>
-  <si>
     <t>1013</t>
   </si>
   <si>
@@ -206,6 +194,18 @@
   </si>
   <si>
     <t>0110241 21 4040</t>
+  </si>
+  <si>
+    <t>1191</t>
+  </si>
+  <si>
+    <t>1012</t>
+  </si>
+  <si>
+    <t>33431020222440</t>
+  </si>
+  <si>
+    <t>40302004403142</t>
   </si>
 </sst>
 </file>
@@ -600,7 +600,7 @@
         <v>7</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -611,7 +611,7 @@
         <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -627,76 +627,76 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>23</v>
-      </c>
       <c r="C9" s="1" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>27</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>12</v>
@@ -704,79 +704,79 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
utf-8 encoding and minor safeguard to addstarstocorrectchoices
</commit_message>
<xml_diff>
--- a/All.xlsx
+++ b/All.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\souri\Dropbox\Machinegrading\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EAEF999-9803-4882-BED4-033BE002D23D}" xr6:coauthVersionLast="33" xr6:coauthVersionMax="33" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E18ECB28-94D0-48DA-8155-0BE0169D20E6}" xr6:coauthVersionLast="33" xr6:coauthVersionMax="33" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" xr2:uid="{55B9AD52-30FB-4BC0-874F-7C9A458412C5}"/>
   </bookViews>
@@ -88,9 +88,6 @@
     <t>MUEZZINOGLU MINE</t>
   </si>
   <si>
-    <t>020224011034001</t>
-  </si>
-  <si>
     <t>1014</t>
   </si>
   <si>
@@ -181,31 +178,34 @@
     <t>ACQUAYE AMBER</t>
   </si>
   <si>
-    <t>231001102123440</t>
-  </si>
-  <si>
     <t>413011342023422</t>
   </si>
   <si>
     <t>430244011141021</t>
   </si>
   <si>
-    <t>42022403343402</t>
-  </si>
-  <si>
     <t>0110241 21 4040</t>
   </si>
   <si>
-    <t>1191</t>
-  </si>
-  <si>
     <t>1012</t>
   </si>
   <si>
-    <t>33431020222440</t>
-  </si>
-  <si>
-    <t>40302004403142</t>
+    <t>334310202224403</t>
+  </si>
+  <si>
+    <t>403020044031422</t>
+  </si>
+  <si>
+    <t>23100110212344</t>
+  </si>
+  <si>
+    <t>420224033434021</t>
+  </si>
+  <si>
+    <t>02022401103400</t>
+  </si>
+  <si>
+    <t>1017</t>
   </si>
 </sst>
 </file>
@@ -600,7 +600,7 @@
         <v>7</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -611,7 +611,7 @@
         <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -633,70 +633,70 @@
         <v>13</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>14</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="C9" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>28</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>12</v>
@@ -704,79 +704,79 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="C13" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>36</v>
-      </c>
       <c r="C16" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="C18" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="C19" s="1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>